<commit_message>
Fragebogen: Einleitung «Beispiele für <Teilbereich>:» statt «Beispiele:»
Wortlaut pro Teilbereich in der Excel (Spalte E) gesetzt, abgeleitet vom Titel;
bei Titeln mit Adjektiv am Anfang klein («Beispiele für berufliche
Kommunikation»). Anzeige erkennt beide Formen. Server- und Offline-Version.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bmaax65xrbFNMF5MHPJVue
</commit_message>
<xml_diff>
--- a/data/items_master.xlsx
+++ b/data/items_master.xlsx
@@ -977,15 +977,15 @@
   <dimension ref="A1:I133"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="10" customWidth="1" style="39" min="1" max="1"/>
-    <col width="28" customWidth="1" style="39" min="2" max="2"/>
-    <col width="6" customWidth="1" style="39" min="3" max="3"/>
-    <col width="34" customWidth="1" style="39" min="4" max="4"/>
-    <col width="7" customWidth="1" style="39" min="5" max="5"/>
-    <col width="16" customWidth="1" style="39" min="6" max="6"/>
-    <col width="100" customWidth="1" style="39" min="7" max="7"/>
-    <col width="72" customWidth="1" style="39" min="8" max="8"/>
-    <col width="60" customWidth="1" style="39" min="9" max="9"/>
+    <col width="10" customWidth="1" style="87" min="1" max="1"/>
+    <col width="28" customWidth="1" style="87" min="2" max="2"/>
+    <col width="6" customWidth="1" style="87" min="3" max="3"/>
+    <col width="34" customWidth="1" style="87" min="4" max="4"/>
+    <col width="7" customWidth="1" style="87" min="5" max="5"/>
+    <col width="16" customWidth="1" style="87" min="6" max="6"/>
+    <col width="100" customWidth="1" style="87" min="7" max="7"/>
+    <col width="72" customWidth="1" style="87" min="8" max="8"/>
+    <col width="60" customWidth="1" style="87" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26.25" customHeight="1" s="40">
@@ -10403,8 +10403,8 @@
   <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="22" customWidth="1" style="39" min="1" max="1"/>
-    <col width="100" customWidth="1" style="39" min="2" max="2"/>
+    <col width="22" customWidth="1" style="87" min="1" max="1"/>
+    <col width="100" customWidth="1" style="87" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="40">
@@ -10414,6 +10414,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="40">
       <c r="A3" s="49" t="inlineStr">
         <is>
@@ -10474,6 +10475,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="64.90000000000001" customHeight="1" s="40">
       <c r="A9" s="49" t="inlineStr">
         <is>
@@ -10534,6 +10536,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="40">
       <c r="A15" s="49" t="inlineStr">
         <is>
@@ -10606,6 +10609,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="15" customHeight="1" s="40">
       <c r="A22" s="49" t="inlineStr">
         <is>
@@ -10656,13 +10660,13 @@
   <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="10" customWidth="1" style="39" min="1" max="1"/>
-    <col width="7" customWidth="1" style="39" min="2" max="2"/>
-    <col width="18" customWidth="1" style="39" min="3" max="3"/>
-    <col width="110" customWidth="1" style="39" min="4" max="4"/>
-    <col width="72" customWidth="1" style="39" min="5" max="5"/>
-    <col width="9" customWidth="1" style="39" min="6" max="6"/>
-    <col width="11" customWidth="1" style="39" min="7" max="7"/>
+    <col width="10" customWidth="1" style="87" min="1" max="1"/>
+    <col width="7" customWidth="1" style="87" min="2" max="2"/>
+    <col width="18" customWidth="1" style="87" min="3" max="3"/>
+    <col width="110" customWidth="1" style="87" min="4" max="4"/>
+    <col width="72" customWidth="1" style="87" min="5" max="5"/>
+    <col width="9" customWidth="1" style="87" min="6" max="6"/>
+    <col width="11" customWidth="1" style="87" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="40">
@@ -10672,6 +10676,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="40">
       <c r="A3" s="53" t="inlineStr">
         <is>
@@ -10720,7 +10725,7 @@
       <c r="D4" s="55" t="n"/>
       <c r="E4" s="56" t="inlineStr">
         <is>
-          <t>Beispiele: E-Mail, Schulportal, Messenger der Schule, Elternkommunikation, Videokonferenz</t>
+          <t>Beispiele für berufliche Kommunikation: E-Mail, Schulportal, Messenger der Schule, Elternkommunikation, Videokonferenz</t>
         </is>
       </c>
     </row>
@@ -11115,6 +11120,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="30" customHeight="1" s="40">
       <c r="A12" s="54" t="inlineStr">
         <is>
@@ -11126,7 +11132,7 @@
       <c r="D12" s="55" t="n"/>
       <c r="E12" s="56" t="inlineStr">
         <is>
-          <t>Beispiele: gemeinsame Ablage, Online-Plattform, Videokonferenz, Online-Communities für Lehrpersonen</t>
+          <t>Beispiele für kollegiale Zusammenarbeit: gemeinsame Ablage, Online-Plattform, Videokonferenz, Online-Communities für Lehrpersonen</t>
         </is>
       </c>
     </row>
@@ -11502,6 +11508,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1" s="40">
       <c r="A20" s="54" t="inlineStr">
         <is>
@@ -11889,6 +11896,7 @@
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="30" customHeight="1" s="40">
       <c r="A28" s="54" t="inlineStr">
         <is>
@@ -11900,7 +11908,7 @@
       <c r="D28" s="55" t="n"/>
       <c r="E28" s="56" t="inlineStr">
         <is>
-          <t>Beispiele: Online-Kurse, Webinare, Erklärvideos, Fachblogs, Bildungsportale</t>
+          <t>Beispiele für kontinuierliche Weiterentwicklung: Online-Kurse, Webinare, Erklärvideos, Fachblogs, Bildungsportale</t>
         </is>
       </c>
     </row>
@@ -12299,13 +12307,13 @@
   <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="10" customWidth="1" style="39" min="1" max="1"/>
-    <col width="7" customWidth="1" style="39" min="2" max="2"/>
-    <col width="18" customWidth="1" style="39" min="3" max="3"/>
-    <col width="110" customWidth="1" style="39" min="4" max="4"/>
-    <col width="72" customWidth="1" style="39" min="5" max="5"/>
-    <col width="9" customWidth="1" style="39" min="6" max="6"/>
-    <col width="11" customWidth="1" style="39" min="7" max="7"/>
+    <col width="10" customWidth="1" style="87" min="1" max="1"/>
+    <col width="7" customWidth="1" style="87" min="2" max="2"/>
+    <col width="18" customWidth="1" style="87" min="3" max="3"/>
+    <col width="110" customWidth="1" style="87" min="4" max="4"/>
+    <col width="72" customWidth="1" style="87" min="5" max="5"/>
+    <col width="9" customWidth="1" style="87" min="6" max="6"/>
+    <col width="11" customWidth="1" style="87" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="40">
@@ -12315,6 +12323,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="40">
       <c r="A3" s="60" t="inlineStr">
         <is>
@@ -12363,7 +12372,7 @@
       <c r="D4" s="62" t="n"/>
       <c r="E4" s="63" t="inlineStr">
         <is>
-          <t>Beispiele: Arbeitsblätter, Lernvideos, Online-Quiz, Bildungsplattformen, offene Lernmaterialien (OER)</t>
+          <t>Beispiele für Auswählen digitaler Ressourcen: Arbeitsblätter, Lernvideos, Online-Quiz, Bildungsplattformen, offene Lernmaterialien (OER)</t>
         </is>
       </c>
     </row>
@@ -12739,6 +12748,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="30" customHeight="1" s="40">
       <c r="A12" s="61" t="inlineStr">
         <is>
@@ -12750,7 +12760,7 @@
       <c r="D12" s="62" t="n"/>
       <c r="E12" s="63" t="inlineStr">
         <is>
-          <t>Beispiele: Präsentationen, interaktive Übungen, Erklärvideos, Lernpfade, digitale Lernumgebungen</t>
+          <t>Beispiele für Erstellen und Anpassen digitaler Ressourcen: Präsentationen, interaktive Übungen, Erklärvideos, Lernpfade, digitale Lernumgebungen</t>
         </is>
       </c>
     </row>
@@ -13126,6 +13136,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1" s="40">
       <c r="A20" s="61" t="inlineStr">
         <is>
@@ -13137,7 +13148,7 @@
       <c r="D20" s="62" t="n"/>
       <c r="E20" s="63" t="inlineStr">
         <is>
-          <t>Beispiele: Ablage in der Cloud, Links teilen, Lernplattform, Urheberrecht, Schutz von Personendaten</t>
+          <t>Beispiele für Organisieren, Schützen und Teilen digitaler Ressourcen: Ablage in der Cloud, Links teilen, Lernplattform, Urheberrecht, Schutz von Personendaten</t>
         </is>
       </c>
     </row>
@@ -13535,13 +13546,13 @@
   <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="10" customWidth="1" style="39" min="1" max="1"/>
-    <col width="7" customWidth="1" style="39" min="2" max="2"/>
-    <col width="18" customWidth="1" style="39" min="3" max="3"/>
-    <col width="110" customWidth="1" style="39" min="4" max="4"/>
-    <col width="72" customWidth="1" style="39" min="5" max="5"/>
-    <col width="9" customWidth="1" style="39" min="6" max="6"/>
-    <col width="11" customWidth="1" style="39" min="7" max="7"/>
+    <col width="10" customWidth="1" style="87" min="1" max="1"/>
+    <col width="7" customWidth="1" style="87" min="2" max="2"/>
+    <col width="18" customWidth="1" style="87" min="3" max="3"/>
+    <col width="110" customWidth="1" style="87" min="4" max="4"/>
+    <col width="72" customWidth="1" style="87" min="5" max="5"/>
+    <col width="9" customWidth="1" style="87" min="6" max="6"/>
+    <col width="11" customWidth="1" style="87" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="40">
@@ -13551,6 +13562,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="40">
       <c r="A3" s="65" t="inlineStr">
         <is>
@@ -13599,7 +13611,7 @@
       <c r="D4" s="67" t="n"/>
       <c r="E4" s="68" t="inlineStr">
         <is>
-          <t>Beispiele: Apps, Lernplattform, interaktive Wandtafel, Simulationen, Tools für die Zusammenarbeit</t>
+          <t>Beispiele für Lehren: Apps, Lernplattform, interaktive Wandtafel, Simulationen, Tools für die Zusammenarbeit</t>
         </is>
       </c>
     </row>
@@ -14013,6 +14025,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="30" customHeight="1" s="40">
       <c r="A12" s="66" t="inlineStr">
         <is>
@@ -14024,7 +14037,7 @@
       <c r="D12" s="67" t="n"/>
       <c r="E12" s="68" t="inlineStr">
         <is>
-          <t>Beispiele: automatisches Feedback, Chat, Umfrage, gemeinsames Online-Dokument, Lernverlauf auf der Plattform</t>
+          <t>Beispiele für Lernbegleitung: automatisches Feedback, Chat, Umfrage, gemeinsames Online-Dokument, Lernverlauf auf der Plattform</t>
         </is>
       </c>
     </row>
@@ -14400,6 +14413,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1" s="40">
       <c r="A20" s="66" t="inlineStr">
         <is>
@@ -14411,7 +14425,7 @@
       <c r="D20" s="67" t="n"/>
       <c r="E20" s="68" t="inlineStr">
         <is>
-          <t>Beispiele: gemeinsame Online-Dokumente, Forum, Wiki, Projektplattform, virtueller Austausch</t>
+          <t>Beispiele für kollaboratives Lernen: gemeinsame Online-Dokumente, Forum, Wiki, Projektplattform, virtueller Austausch</t>
         </is>
       </c>
     </row>
@@ -14787,6 +14801,7 @@
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="30" customHeight="1" s="40">
       <c r="A28" s="66" t="inlineStr">
         <is>
@@ -14798,7 +14813,7 @@
       <c r="D28" s="67" t="n"/>
       <c r="E28" s="68" t="inlineStr">
         <is>
-          <t>Beispiele: digitaler Lernplan, Lernjournal, Fortschrittsanzeige, E-Portfolio, Lernplattform</t>
+          <t>Beispiele für selbstgesteuertes Lernen: digitaler Lernplan, Lernjournal, Fortschrittsanzeige, E-Portfolio, Lernplattform</t>
         </is>
       </c>
     </row>
@@ -15197,13 +15212,13 @@
   <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="10" customWidth="1" style="39" min="1" max="1"/>
-    <col width="7" customWidth="1" style="39" min="2" max="2"/>
-    <col width="18" customWidth="1" style="39" min="3" max="3"/>
-    <col width="110" customWidth="1" style="39" min="4" max="4"/>
-    <col width="72" customWidth="1" style="39" min="5" max="5"/>
-    <col width="9" customWidth="1" style="39" min="6" max="6"/>
-    <col width="11" customWidth="1" style="39" min="7" max="7"/>
+    <col width="10" customWidth="1" style="87" min="1" max="1"/>
+    <col width="7" customWidth="1" style="87" min="2" max="2"/>
+    <col width="18" customWidth="1" style="87" min="3" max="3"/>
+    <col width="110" customWidth="1" style="87" min="4" max="4"/>
+    <col width="72" customWidth="1" style="87" min="5" max="5"/>
+    <col width="9" customWidth="1" style="87" min="6" max="6"/>
+    <col width="11" customWidth="1" style="87" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="40">
@@ -15213,6 +15228,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="40">
       <c r="A3" s="70" t="inlineStr">
         <is>
@@ -15261,7 +15277,7 @@
       <c r="D4" s="72" t="n"/>
       <c r="E4" s="73" t="inlineStr">
         <is>
-          <t>Beispiele: Quiz, Online-Umfrage, digitaler Test, Bewertungsraster, E-Portfolio, Peer-Feedback</t>
+          <t>Beispiele für Lernstandserhebung: Quiz, Online-Umfrage, digitaler Test, Bewertungsraster, E-Portfolio, Peer-Feedback</t>
         </is>
       </c>
     </row>
@@ -15656,6 +15672,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="30" customHeight="1" s="40">
       <c r="A12" s="71" t="inlineStr">
         <is>
@@ -15667,7 +15684,7 @@
       <c r="D12" s="72" t="n"/>
       <c r="E12" s="73" t="inlineStr">
         <is>
-          <t>Beispiele: Quiz, Bearbeitungsstand auf der Lernplattform, Umfrage, Auswertung in Tabellen, Learning Analytics</t>
+          <t>Beispiele für Analyse der Lernevidenz: Quiz, Bearbeitungsstand auf der Lernplattform, Umfrage, Auswertung in Tabellen, Learning Analytics</t>
         </is>
       </c>
     </row>
@@ -16043,6 +16060,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1" s="40">
       <c r="A20" s="71" t="inlineStr">
         <is>
@@ -16054,7 +16072,7 @@
       <c r="D20" s="72" t="n"/>
       <c r="E20" s="73" t="inlineStr">
         <is>
-          <t>Beispiele: Online-Übungen mit automatischer Rückmeldung, digitale Kommentare, Peer-Feedback, Umfragen</t>
+          <t>Beispiele für Feedback und Planung: Online-Übungen mit automatischer Rückmeldung, digitale Kommentare, Peer-Feedback, Umfragen</t>
         </is>
       </c>
     </row>
@@ -16452,13 +16470,13 @@
   <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="10" customWidth="1" style="39" min="1" max="1"/>
-    <col width="7" customWidth="1" style="39" min="2" max="2"/>
-    <col width="18" customWidth="1" style="39" min="3" max="3"/>
-    <col width="110" customWidth="1" style="39" min="4" max="4"/>
-    <col width="72" customWidth="1" style="39" min="5" max="5"/>
-    <col width="9" customWidth="1" style="39" min="6" max="6"/>
-    <col width="11" customWidth="1" style="39" min="7" max="7"/>
+    <col width="10" customWidth="1" style="87" min="1" max="1"/>
+    <col width="7" customWidth="1" style="87" min="2" max="2"/>
+    <col width="18" customWidth="1" style="87" min="3" max="3"/>
+    <col width="110" customWidth="1" style="87" min="4" max="4"/>
+    <col width="72" customWidth="1" style="87" min="5" max="5"/>
+    <col width="9" customWidth="1" style="87" min="6" max="6"/>
+    <col width="11" customWidth="1" style="87" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="40">
@@ -16468,6 +16486,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="40">
       <c r="A3" s="75" t="inlineStr">
         <is>
@@ -16516,7 +16535,7 @@
       <c r="D4" s="77" t="n"/>
       <c r="E4" s="78" t="inlineStr">
         <is>
-          <t>Beispiele: Zugang zu Geräten und Internet, Vorlesefunktion, einfache Sprache, barrierefreie Dokumente</t>
+          <t>Beispiele für Barrierefreiheit und digitale Teilhabe: Zugang zu Geräten und Internet, Vorlesefunktion, einfache Sprache, barrierefreie Dokumente</t>
         </is>
       </c>
     </row>
@@ -16892,6 +16911,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="30" customHeight="1" s="40">
       <c r="A12" s="76" t="inlineStr">
         <is>
@@ -16903,7 +16923,7 @@
       <c r="D12" s="77" t="n"/>
       <c r="E12" s="78" t="inlineStr">
         <is>
-          <t>Beispiele: Aufgaben auf verschiedenen Niveaus, adaptive Übungsprogramme, Lernpfade, individuelle Lernpläne</t>
+          <t>Beispiele für Differenzierung: Aufgaben auf verschiedenen Niveaus, adaptive Übungsprogramme, Lernpfade, individuelle Lernpläne</t>
         </is>
       </c>
     </row>
@@ -17279,6 +17299,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1" s="40">
       <c r="A20" s="76" t="inlineStr">
         <is>
@@ -17290,7 +17311,7 @@
       <c r="D20" s="77" t="n"/>
       <c r="E20" s="78" t="inlineStr">
         <is>
-          <t>Beispiele: Lernspiele, interaktive Übungen, Erklärvideos der Lernenden, Simulationen, Robotik</t>
+          <t>Beispiele für Schüleraktivierung: Lernspiele, interaktive Übungen, Erklärvideos der Lernenden, Simulationen, Robotik</t>
         </is>
       </c>
     </row>
@@ -17688,13 +17709,13 @@
   <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="10" customWidth="1" style="39" min="1" max="1"/>
-    <col width="7" customWidth="1" style="39" min="2" max="2"/>
-    <col width="18" customWidth="1" style="39" min="3" max="3"/>
-    <col width="110" customWidth="1" style="39" min="4" max="4"/>
-    <col width="72" customWidth="1" style="39" min="5" max="5"/>
-    <col width="9" customWidth="1" style="39" min="6" max="6"/>
-    <col width="11" customWidth="1" style="39" min="7" max="7"/>
+    <col width="10" customWidth="1" style="87" min="1" max="1"/>
+    <col width="7" customWidth="1" style="87" min="2" max="2"/>
+    <col width="18" customWidth="1" style="87" min="3" max="3"/>
+    <col width="110" customWidth="1" style="87" min="4" max="4"/>
+    <col width="72" customWidth="1" style="87" min="5" max="5"/>
+    <col width="9" customWidth="1" style="87" min="6" max="6"/>
+    <col width="11" customWidth="1" style="87" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="40">
@@ -17704,6 +17725,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="40">
       <c r="A3" s="80" t="inlineStr">
         <is>
@@ -18128,6 +18150,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="30" customHeight="1" s="40">
       <c r="A12" s="81" t="inlineStr">
         <is>
@@ -18139,7 +18162,7 @@
       <c r="D12" s="82" t="n"/>
       <c r="E12" s="83" t="inlineStr">
         <is>
-          <t>Beispiele: Suchmaschinen und Suchfilter, Quellen vergleichen und zitieren, Diagramme lesen, Falschinformationen erkennen</t>
+          <t>Beispiele für Suchen und Verarbeiten: Suchmaschinen und Suchfilter, Quellen vergleichen und zitieren, Diagramme lesen, Falschinformationen erkennen</t>
         </is>
       </c>
     </row>
@@ -18515,6 +18538,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="30" customHeight="1" s="40">
       <c r="A20" s="81" t="inlineStr">
         <is>
@@ -18526,7 +18550,7 @@
       <c r="D20" s="82" t="n"/>
       <c r="E20" s="83" t="inlineStr">
         <is>
-          <t>Beispiele: Klassenchat, Online-Meeting, gemeinsame Dokumente, Netiquette, Peer-Feedback, Online-Diskussion</t>
+          <t>Beispiele für Kommunizieren und Kooperieren: Klassenchat, Online-Meeting, gemeinsame Dokumente, Netiquette, Peer-Feedback, Online-Diskussion</t>
         </is>
       </c>
     </row>
@@ -18902,6 +18926,7 @@
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="30" customHeight="1" s="40">
       <c r="A28" s="81" t="inlineStr">
         <is>
@@ -18913,7 +18938,7 @@
       <c r="D28" s="82" t="n"/>
       <c r="E28" s="83" t="inlineStr">
         <is>
-          <t>Beispiele: Texte, Fotos, Präsentationen, Audio und Video, digitale Geschichten, Blog, E-Portfolio</t>
+          <t>Beispiele für Produzieren und Präsentieren: Texte, Fotos, Präsentationen, Audio und Video, digitale Geschichten, Blog, E-Portfolio</t>
         </is>
       </c>
     </row>
@@ -19289,6 +19314,7 @@
         <v/>
       </c>
     </row>
+    <row r="35"/>
     <row r="36" ht="30" customHeight="1" s="40">
       <c r="A36" s="81" t="inlineStr">
         <is>
@@ -19300,7 +19326,7 @@
       <c r="D36" s="82" t="n"/>
       <c r="E36" s="83" t="inlineStr">
         <is>
-          <t>Beispiele: Datenschutz, Urheberrecht, App-Berechtigungen, Fake News, digitaler Fussabdruck</t>
+          <t>Beispiele für Analysieren und Reflektieren: Datenschutz, Urheberrecht, App-Berechtigungen, Fake News, digitaler Fussabdruck</t>
         </is>
       </c>
     </row>

</xml_diff>